<commit_message>
Improve MP2027 audit dashboard and data parsers
</commit_message>
<xml_diff>
--- a/OUTPUT_FY2027/MP_CC_1412000006.xlsx
+++ b/OUTPUT_FY2027/MP_CC_1412000006.xlsx
@@ -17761,18 +17761,54 @@
         <v/>
       </c>
       <c r="E36" s="244" t="n"/>
-      <c r="F36" s="193" t="n"/>
-      <c r="G36" s="246" t="n"/>
-      <c r="H36" s="246" t="n"/>
-      <c r="I36" s="246" t="n"/>
-      <c r="J36" s="246" t="n"/>
-      <c r="K36" s="246" t="n"/>
-      <c r="L36" s="246" t="n"/>
-      <c r="M36" s="246" t="n"/>
-      <c r="N36" s="246" t="n"/>
-      <c r="O36" s="246" t="n"/>
-      <c r="P36" s="246" t="n"/>
-      <c r="Q36" s="246" t="n"/>
+      <c r="F36" s="193">
+        <f>ROUND(244.09*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="G36" s="246">
+        <f>ROUND(245.37*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="H36" s="246">
+        <f>ROUND(283.68*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="I36" s="246">
+        <f>ROUND(275.75*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="J36" s="246">
+        <f>ROUND(266.32*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="K36" s="246">
+        <f>ROUND(270.12*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="L36" s="246">
+        <f>ROUND(276.59*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="M36" s="246">
+        <f>ROUND(273.85*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="N36" s="246">
+        <f>ROUND(272.09*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="O36" s="246">
+        <f>ROUND(271.55*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="P36" s="246">
+        <f>ROUND(254.83*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="Q36" s="246">
+        <f>ROUND(277.02*$B$2,0)</f>
+        <v/>
+      </c>
       <c r="R36" s="199">
         <f>SUM(F36:Q36)</f>
         <v/>
@@ -17801,18 +17837,54 @@
         <v/>
       </c>
       <c r="E37" s="244" t="n"/>
-      <c r="F37" s="193" t="n"/>
-      <c r="G37" s="246" t="n"/>
-      <c r="H37" s="246" t="n"/>
-      <c r="I37" s="246" t="n"/>
-      <c r="J37" s="246" t="n"/>
-      <c r="K37" s="246" t="n"/>
-      <c r="L37" s="246" t="n"/>
-      <c r="M37" s="246" t="n"/>
-      <c r="N37" s="246" t="n"/>
-      <c r="O37" s="246" t="n"/>
-      <c r="P37" s="246" t="n"/>
-      <c r="Q37" s="246" t="n"/>
+      <c r="F37" s="193">
+        <f>ROUND(16.48*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="G37" s="246">
+        <f>ROUND(16.56*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="H37" s="246">
+        <f>ROUND(19.15*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="I37" s="246">
+        <f>ROUND(18.61*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="J37" s="246">
+        <f>ROUND(17.98*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="K37" s="246">
+        <f>ROUND(18.23*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="L37" s="246">
+        <f>ROUND(18.67*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="M37" s="246">
+        <f>ROUND(18.48*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="N37" s="246">
+        <f>ROUND(18.37*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="O37" s="246">
+        <f>ROUND(18.33*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="P37" s="246">
+        <f>ROUND(17.2*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="Q37" s="246">
+        <f>ROUND(18.7*$B$2,0)</f>
+        <v/>
+      </c>
       <c r="R37" s="199">
         <f>SUM(F37:Q37)</f>
         <v/>
@@ -17904,7 +17976,7 @@
     <row r="40" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A40" s="225" t="n"/>
       <c r="B40" s="179" t="n">
-        <v>5005066281</v>
+        <v>9114120007</v>
       </c>
       <c r="C40" s="182">
         <f>IFERROR(IF(VLOOKUP($B40,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B40,勘定科目!$A:$E,2,0)),"")</f>
@@ -17915,41 +17987,53 @@
         <v/>
       </c>
       <c r="E40" s="244" t="n"/>
-      <c r="F40" s="193" t="n">
-        <v>932009</v>
-      </c>
-      <c r="G40" s="246" t="n">
-        <v>1158252</v>
-      </c>
-      <c r="H40" s="246" t="n">
-        <v>1702420</v>
-      </c>
-      <c r="I40" s="246" t="n">
-        <v>2125161</v>
-      </c>
-      <c r="J40" s="246" t="n">
-        <v>2211909</v>
-      </c>
-      <c r="K40" s="246" t="n">
-        <v>2026479</v>
-      </c>
-      <c r="L40" s="246" t="n">
-        <v>1790128</v>
-      </c>
-      <c r="M40" s="246" t="n">
-        <v>1500861</v>
-      </c>
-      <c r="N40" s="246" t="n">
-        <v>1070755</v>
-      </c>
-      <c r="O40" s="246" t="n">
-        <v>923989</v>
-      </c>
-      <c r="P40" s="246" t="n">
-        <v>842827</v>
-      </c>
-      <c r="Q40" s="246" t="n">
-        <v>821816</v>
+      <c r="F40" s="193">
+        <f>ROUND(156.9*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="G40" s="246">
+        <f>ROUND(148.89*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="H40" s="246">
+        <f>ROUND(172.13*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="I40" s="246">
+        <f>ROUND(167.32*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="J40" s="246">
+        <f>ROUND(161.6*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="K40" s="246">
+        <f>ROUND(163.9*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="L40" s="246">
+        <f>ROUND(167.83*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="M40" s="246">
+        <f>ROUND(166.17*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="N40" s="246">
+        <f>ROUND(165.1*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="O40" s="246">
+        <f>ROUND(164.77*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="P40" s="246">
+        <f>ROUND(154.62*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="Q40" s="246">
+        <f>ROUND(168.09*$B$2,0)</f>
+        <v/>
       </c>
       <c r="R40" s="199">
         <f>SUM(F40:Q40)</f>
@@ -17968,7 +18052,7 @@
     <row r="41" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A41" s="225" t="n"/>
       <c r="B41" s="179" t="n">
-        <v>5005066282</v>
+        <v>9114120007</v>
       </c>
       <c r="C41" s="182">
         <f>IFERROR(IF(VLOOKUP($B41,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B41,勘定科目!$A:$E,2,0)),"")</f>
@@ -17979,41 +18063,53 @@
         <v/>
       </c>
       <c r="E41" s="244" t="n"/>
-      <c r="F41" s="193" t="n">
-        <v>647376</v>
-      </c>
-      <c r="G41" s="246" t="n">
-        <v>705438</v>
-      </c>
-      <c r="H41" s="246" t="n">
-        <v>986242</v>
-      </c>
-      <c r="I41" s="246" t="n">
-        <v>1442423</v>
-      </c>
-      <c r="J41" s="246" t="n">
-        <v>1221608</v>
-      </c>
-      <c r="K41" s="246" t="n">
-        <v>1242901</v>
-      </c>
-      <c r="L41" s="246" t="n">
-        <v>1223902</v>
-      </c>
-      <c r="M41" s="246" t="n">
-        <v>919260</v>
-      </c>
-      <c r="N41" s="246" t="n">
-        <v>902681</v>
-      </c>
-      <c r="O41" s="246" t="n">
-        <v>835389</v>
-      </c>
-      <c r="P41" s="246" t="n">
-        <v>645935</v>
-      </c>
-      <c r="Q41" s="246" t="n">
-        <v>940114</v>
+      <c r="F41" s="193">
+        <f>ROUND(19.89*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="G41" s="246">
+        <f>ROUND(19.4*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="H41" s="246">
+        <f>ROUND(22.43*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="I41" s="246">
+        <f>ROUND(21.8*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="J41" s="246">
+        <f>ROUND(21.06*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="K41" s="246">
+        <f>ROUND(21.36*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="L41" s="246">
+        <f>ROUND(21.87*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="M41" s="246">
+        <f>ROUND(21.65*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="N41" s="246">
+        <f>ROUND(21.51*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="O41" s="246">
+        <f>ROUND(21.47*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="P41" s="246">
+        <f>ROUND(20.15*$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="Q41" s="246">
+        <f>ROUND(21.9*$B$2,0)</f>
+        <v/>
       </c>
       <c r="R41" s="199">
         <f>SUM(F41:Q41)</f>
@@ -18032,7 +18128,7 @@
     <row r="42" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A42" s="225" t="n"/>
       <c r="B42" s="179" t="n">
-        <v>5005056281</v>
+        <v>9114120007</v>
       </c>
       <c r="C42" s="182">
         <f>IFERROR(IF(VLOOKUP($B42,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B42,勘定科目!$A:$E,2,0)),"")</f>
@@ -18043,54 +18139,18 @@
         <v/>
       </c>
       <c r="E42" s="244" t="n"/>
-      <c r="F42" s="193">
-        <f>SUM(F$24:F$25)*39309</f>
-        <v/>
-      </c>
-      <c r="G42" s="193">
-        <f>SUM(F$24:F$25)*37465</f>
-        <v/>
-      </c>
-      <c r="H42" s="193">
-        <f>SUM(G$24:G$25)*43911</f>
-        <v/>
-      </c>
-      <c r="I42" s="193">
-        <f>SUM(H$24:H$25)*46094</f>
-        <v/>
-      </c>
-      <c r="J42" s="193">
-        <f>SUM(I$24:I$25)*37411</f>
-        <v/>
-      </c>
-      <c r="K42" s="193">
-        <f>SUM(J$24:J$25)*40977</f>
-        <v/>
-      </c>
-      <c r="L42" s="193">
-        <f>SUM(K$24:K$25)*43471</f>
-        <v/>
-      </c>
-      <c r="M42" s="193">
-        <f>SUM(L$24:L$25)*42228</f>
-        <v/>
-      </c>
-      <c r="N42" s="193">
-        <f>SUM(M$24:M$25)*43136</f>
-        <v/>
-      </c>
-      <c r="O42" s="193">
-        <f>SUM(N$24:N$25)*39648</f>
-        <v/>
-      </c>
-      <c r="P42" s="193">
-        <f>SUM(O$24:O$25)*24211</f>
-        <v/>
-      </c>
-      <c r="Q42" s="193">
-        <f>SUM(P$24:P$25)*44420</f>
-        <v/>
-      </c>
+      <c r="F42" s="193" t="n"/>
+      <c r="G42" s="193" t="n"/>
+      <c r="H42" s="193" t="n"/>
+      <c r="I42" s="193" t="n"/>
+      <c r="J42" s="193" t="n"/>
+      <c r="K42" s="193" t="n"/>
+      <c r="L42" s="193" t="n"/>
+      <c r="M42" s="193" t="n"/>
+      <c r="N42" s="193" t="n"/>
+      <c r="O42" s="193" t="n"/>
+      <c r="P42" s="193" t="n"/>
+      <c r="Q42" s="193" t="n"/>
       <c r="R42" s="199">
         <f>SUM(F42:Q42)</f>
         <v/>
@@ -18136,7 +18196,7 @@
     <row r="44" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A44" s="225" t="n"/>
       <c r="B44" s="179" t="n">
-        <v>5005246286</v>
+        <v>5005066281</v>
       </c>
       <c r="C44" s="182">
         <f>IFERROR(IF(VLOOKUP($B44,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B44,勘定科目!$A:$E,2,0)),"")</f>
@@ -18148,51 +18208,51 @@
       </c>
       <c r="E44" s="244" t="n"/>
       <c r="F44" s="193">
-        <f>SUM(F$24:F$25)*58682</f>
+        <f>932009</f>
         <v/>
       </c>
       <c r="G44" s="246">
-        <f>SUM(F$24:F$25)*60231</f>
+        <f>1158252</f>
         <v/>
       </c>
       <c r="H44" s="246">
-        <f>SUM(G$24:G$25)*65552</f>
+        <f>1702420</f>
         <v/>
       </c>
       <c r="I44" s="246">
-        <f>SUM(H$24:H$25)*60210</f>
+        <f>2125161</f>
         <v/>
       </c>
       <c r="J44" s="246">
-        <f>SUM(I$24:I$25)*55849</f>
+        <f>2211909</f>
         <v/>
       </c>
       <c r="K44" s="246">
-        <f>SUM(J$24:J$25)*57094</f>
+        <f>2026479</f>
         <v/>
       </c>
       <c r="L44" s="246">
-        <f>SUM(K$24:K$25)*60568</f>
+        <f>1790128</f>
         <v/>
       </c>
       <c r="M44" s="246">
-        <f>SUM(L$24:L$25)*58837</f>
+        <f>1500861</f>
         <v/>
       </c>
       <c r="N44" s="246">
-        <f>SUM(M$24:M$25)*58163</f>
+        <f>1070755</f>
         <v/>
       </c>
       <c r="O44" s="246">
-        <f>SUM(N$24:N$25)*55242</f>
+        <f>923989</f>
         <v/>
       </c>
       <c r="P44" s="246">
-        <f>SUM(O$24:O$25)*46000</f>
+        <f>842827</f>
         <v/>
       </c>
       <c r="Q44" s="246">
-        <f>SUM(P$24:P$25)*58022</f>
+        <f>821816</f>
         <v/>
       </c>
       <c r="R44" s="199">
@@ -18223,18 +18283,54 @@
         <v/>
       </c>
       <c r="E45" s="244" t="n"/>
-      <c r="F45" s="193" t="n"/>
-      <c r="G45" s="246" t="n"/>
-      <c r="H45" s="246" t="n"/>
-      <c r="I45" s="246" t="n"/>
-      <c r="J45" s="246" t="n"/>
-      <c r="K45" s="246" t="n"/>
-      <c r="L45" s="246" t="n"/>
-      <c r="M45" s="246" t="n"/>
-      <c r="N45" s="246" t="n"/>
-      <c r="O45" s="246" t="n"/>
-      <c r="P45" s="246" t="n"/>
-      <c r="Q45" s="246" t="n"/>
+      <c r="F45" s="193">
+        <f>647376</f>
+        <v/>
+      </c>
+      <c r="G45" s="246">
+        <f>705438</f>
+        <v/>
+      </c>
+      <c r="H45" s="246">
+        <f>986242</f>
+        <v/>
+      </c>
+      <c r="I45" s="246">
+        <f>1442423</f>
+        <v/>
+      </c>
+      <c r="J45" s="246">
+        <f>1221608</f>
+        <v/>
+      </c>
+      <c r="K45" s="246">
+        <f>1242901</f>
+        <v/>
+      </c>
+      <c r="L45" s="246">
+        <f>1223902</f>
+        <v/>
+      </c>
+      <c r="M45" s="246">
+        <f>919260</f>
+        <v/>
+      </c>
+      <c r="N45" s="246">
+        <f>902681</f>
+        <v/>
+      </c>
+      <c r="O45" s="246">
+        <f>835389</f>
+        <v/>
+      </c>
+      <c r="P45" s="246">
+        <f>645935</f>
+        <v/>
+      </c>
+      <c r="Q45" s="246">
+        <f>940114</f>
+        <v/>
+      </c>
       <c r="R45" s="199">
         <f>SUM(F45:Q45)</f>
         <v/>
@@ -18252,7 +18348,7 @@
     <row r="46" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A46" s="225" t="n"/>
       <c r="B46" s="179" t="n">
-        <v>5006016260</v>
+        <v>5005056281</v>
       </c>
       <c r="C46" s="182">
         <f>IFERROR(IF(VLOOKUP($B46,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B46,勘定科目!$A:$E,2,0)),"")</f>
@@ -18264,51 +18360,51 @@
       </c>
       <c r="E46" s="244" t="n"/>
       <c r="F46" s="193">
-        <f>ROUND(244.09*$B$2,0)</f>
+        <f>SUM(F$24:F$25)*39309</f>
         <v/>
       </c>
       <c r="G46" s="246">
-        <f>ROUND(245.37*$B$2,0)</f>
+        <f>SUM(F$24:F$25)*37465</f>
         <v/>
       </c>
       <c r="H46" s="246">
-        <f>ROUND(283.68*$B$2,0)</f>
+        <f>SUM(G$24:G$25)*43911</f>
         <v/>
       </c>
       <c r="I46" s="246">
-        <f>ROUND(275.75*$B$2,0)</f>
+        <f>SUM(H$24:H$25)*46094</f>
         <v/>
       </c>
       <c r="J46" s="246">
-        <f>ROUND(266.32*$B$2,0)</f>
+        <f>SUM(I$24:I$25)*37411</f>
         <v/>
       </c>
       <c r="K46" s="246">
-        <f>ROUND(270.12*$B$2,0)</f>
+        <f>SUM(J$24:J$25)*40977</f>
         <v/>
       </c>
       <c r="L46" s="246">
-        <f>ROUND(276.59*$B$2,0)</f>
+        <f>SUM(K$24:K$25)*43471</f>
         <v/>
       </c>
       <c r="M46" s="246">
-        <f>ROUND(273.85*$B$2,0)</f>
+        <f>SUM(L$24:L$25)*42228</f>
         <v/>
       </c>
       <c r="N46" s="246">
-        <f>ROUND(272.09*$B$2,0)</f>
+        <f>SUM(M$24:M$25)*43136</f>
         <v/>
       </c>
       <c r="O46" s="246">
-        <f>ROUND(271.55*$B$2,0)</f>
+        <f>SUM(N$24:N$25)*39648</f>
         <v/>
       </c>
       <c r="P46" s="246">
-        <f>ROUND(254.83*$B$2,0)</f>
+        <f>SUM(O$24:O$25)*24211</f>
         <v/>
       </c>
       <c r="Q46" s="246">
-        <f>ROUND(277.02*$B$2,0)</f>
+        <f>SUM(P$24:P$25)*44420</f>
         <v/>
       </c>
       <c r="R46" s="199">
@@ -18327,9 +18423,7 @@
     </row>
     <row r="47" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A47" s="225" t="n"/>
-      <c r="B47" s="179" t="n">
-        <v>5006016261</v>
-      </c>
+      <c r="B47" s="179" t="n"/>
       <c r="C47" s="182">
         <f>IFERROR(IF(VLOOKUP($B47,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B47,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18339,54 +18433,18 @@
         <v/>
       </c>
       <c r="E47" s="244" t="n"/>
-      <c r="F47" s="193">
-        <f>ROUND(16.48*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="G47" s="246">
-        <f>ROUND(16.56*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="H47" s="246">
-        <f>ROUND(19.15*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="I47" s="246">
-        <f>ROUND(18.61*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="J47" s="246">
-        <f>ROUND(17.98*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="K47" s="246">
-        <f>ROUND(18.23*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="L47" s="246">
-        <f>ROUND(18.67*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="M47" s="246">
-        <f>ROUND(18.48*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="N47" s="246">
-        <f>ROUND(18.37*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="O47" s="246">
-        <f>ROUND(18.33*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="P47" s="246">
-        <f>ROUND(17.2*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="Q47" s="246">
-        <f>ROUND(18.7*$B$2,0)</f>
-        <v/>
-      </c>
+      <c r="F47" s="193" t="n"/>
+      <c r="G47" s="246" t="n"/>
+      <c r="H47" s="246" t="n"/>
+      <c r="I47" s="246" t="n"/>
+      <c r="J47" s="246" t="n"/>
+      <c r="K47" s="246" t="n"/>
+      <c r="L47" s="246" t="n"/>
+      <c r="M47" s="246" t="n"/>
+      <c r="N47" s="246" t="n"/>
+      <c r="O47" s="246" t="n"/>
+      <c r="P47" s="246" t="n"/>
+      <c r="Q47" s="246" t="n"/>
       <c r="R47" s="199">
         <f>SUM(F47:Q47)</f>
         <v/>
@@ -18400,7 +18458,7 @@
     <row r="48" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A48" s="225" t="n"/>
       <c r="B48" s="179" t="n">
-        <v>5006016244</v>
+        <v>5005016372</v>
       </c>
       <c r="C48" s="182">
         <f>IFERROR(IF(VLOOKUP($B48,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B48,勘定科目!$A:$E,2,0)),"")</f>
@@ -18411,18 +18469,54 @@
         <v/>
       </c>
       <c r="E48" s="244" t="n"/>
-      <c r="F48" s="193" t="n"/>
-      <c r="G48" s="193" t="n"/>
-      <c r="H48" s="193" t="n"/>
-      <c r="I48" s="193" t="n"/>
-      <c r="J48" s="193" t="n"/>
-      <c r="K48" s="193" t="n"/>
-      <c r="L48" s="193" t="n"/>
-      <c r="M48" s="193" t="n"/>
-      <c r="N48" s="193" t="n"/>
-      <c r="O48" s="193" t="n"/>
-      <c r="P48" s="193" t="n"/>
-      <c r="Q48" s="193" t="n"/>
+      <c r="F48" s="193">
+        <f>SUM(F$24:F$25)*1365</f>
+        <v/>
+      </c>
+      <c r="G48" s="193">
+        <f>SUM(F$24:F$25)*1284</f>
+        <v/>
+      </c>
+      <c r="H48" s="193">
+        <f>SUM(G$24:G$25)*1461</f>
+        <v/>
+      </c>
+      <c r="I48" s="193">
+        <f>SUM(H$24:H$25)*1517</f>
+        <v/>
+      </c>
+      <c r="J48" s="193">
+        <f>SUM(I$24:I$25)*1299</f>
+        <v/>
+      </c>
+      <c r="K48" s="193">
+        <f>SUM(J$24:J$25)*1328</f>
+        <v/>
+      </c>
+      <c r="L48" s="193">
+        <f>SUM(K$24:K$25)*1468</f>
+        <v/>
+      </c>
+      <c r="M48" s="193">
+        <f>SUM(L$24:L$25)*1426</f>
+        <v/>
+      </c>
+      <c r="N48" s="193">
+        <f>SUM(M$24:M$25)*1466</f>
+        <v/>
+      </c>
+      <c r="O48" s="193">
+        <f>SUM(N$24:N$25)*1339</f>
+        <v/>
+      </c>
+      <c r="P48" s="193">
+        <f>SUM(O$24:O$25)*803</f>
+        <v/>
+      </c>
+      <c r="Q48" s="193">
+        <f>SUM(P$24:P$25)*1462</f>
+        <v/>
+      </c>
       <c r="R48" s="199">
         <f>SUM(F48:Q48)</f>
         <v/>
@@ -18451,18 +18545,54 @@
         <v/>
       </c>
       <c r="E49" s="244" t="n"/>
-      <c r="F49" s="193" t="n"/>
-      <c r="G49" s="193" t="n"/>
-      <c r="H49" s="193" t="n"/>
-      <c r="I49" s="193" t="n"/>
-      <c r="J49" s="193" t="n"/>
-      <c r="K49" s="193" t="n"/>
-      <c r="L49" s="193" t="n"/>
-      <c r="M49" s="193" t="n"/>
-      <c r="N49" s="193" t="n"/>
-      <c r="O49" s="193" t="n"/>
-      <c r="P49" s="193" t="n"/>
-      <c r="Q49" s="193" t="n"/>
+      <c r="F49" s="193">
+        <f>SUM(F$24:F$25)*18895</f>
+        <v/>
+      </c>
+      <c r="G49" s="193">
+        <f>SUM(F$24:F$25)*18117</f>
+        <v/>
+      </c>
+      <c r="H49" s="193">
+        <f>SUM(G$24:G$25)*20767</f>
+        <v/>
+      </c>
+      <c r="I49" s="193">
+        <f>SUM(H$24:H$25)*21675</f>
+        <v/>
+      </c>
+      <c r="J49" s="193">
+        <f>SUM(I$24:I$25)*17938</f>
+        <v/>
+      </c>
+      <c r="K49" s="193">
+        <f>SUM(J$24:J$25)*18894</f>
+        <v/>
+      </c>
+      <c r="L49" s="193">
+        <f>SUM(K$24:K$25)*20737</f>
+        <v/>
+      </c>
+      <c r="M49" s="193">
+        <f>SUM(L$24:L$25)*19781</f>
+        <v/>
+      </c>
+      <c r="N49" s="193">
+        <f>SUM(M$24:M$25)*20715</f>
+        <v/>
+      </c>
+      <c r="O49" s="193">
+        <f>SUM(N$24:N$25)*18874</f>
+        <v/>
+      </c>
+      <c r="P49" s="193">
+        <f>SUM(O$24:O$25)*11355</f>
+        <v/>
+      </c>
+      <c r="Q49" s="193">
+        <f>SUM(P$24:P$25)*20665</f>
+        <v/>
+      </c>
       <c r="R49" s="199">
         <f>SUM(F49:Q49)</f>
         <v/>
@@ -18479,60 +18609,22 @@
     </row>
     <row r="50" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A50" s="225" t="n"/>
-      <c r="B50" s="179" t="n">
-        <v>9114120007</v>
-      </c>
+      <c r="B50" s="179" t="n"/>
       <c r="C50" s="182" t="n"/>
       <c r="D50" s="238" t="n"/>
       <c r="E50" s="244" t="n"/>
-      <c r="F50" s="193">
-        <f>ROUND(156.9*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="G50" s="193">
-        <f>ROUND(148.89*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="H50" s="193">
-        <f>ROUND(172.13*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="I50" s="193">
-        <f>ROUND(167.32*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="J50" s="193">
-        <f>ROUND(161.6*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="K50" s="193">
-        <f>ROUND(163.9*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="L50" s="193">
-        <f>ROUND(167.83*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="M50" s="193">
-        <f>ROUND(166.17*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="N50" s="193">
-        <f>ROUND(165.1*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="O50" s="193">
-        <f>ROUND(164.77*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="P50" s="193">
-        <f>ROUND(154.62*$B$2,0)</f>
-        <v/>
-      </c>
-      <c r="Q50" s="193">
-        <f>ROUND(168.09*$B$2,0)</f>
-        <v/>
-      </c>
+      <c r="F50" s="193" t="n"/>
+      <c r="G50" s="193" t="n"/>
+      <c r="H50" s="193" t="n"/>
+      <c r="I50" s="193" t="n"/>
+      <c r="J50" s="193" t="n"/>
+      <c r="K50" s="193" t="n"/>
+      <c r="L50" s="193" t="n"/>
+      <c r="M50" s="193" t="n"/>
+      <c r="N50" s="193" t="n"/>
+      <c r="O50" s="193" t="n"/>
+      <c r="P50" s="193" t="n"/>
+      <c r="Q50" s="193" t="n"/>
       <c r="R50" s="199">
         <f>SUM(F50:Q50)</f>
         <v/>
@@ -18546,7 +18638,7 @@
     <row r="51" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A51" s="225" t="n"/>
       <c r="B51" s="179" t="n">
-        <v>9114120007</v>
+        <v>5005246286</v>
       </c>
       <c r="C51" s="182">
         <f>IFERROR(IF(VLOOKUP($B51,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B51,勘定科目!$A:$E,2,0)),"")</f>
@@ -18558,51 +18650,51 @@
       </c>
       <c r="E51" s="244" t="n"/>
       <c r="F51" s="193">
-        <f>ROUND(19.89*$B$2,0)</f>
+        <f>SUM(F$24:F$25)*58682</f>
         <v/>
       </c>
       <c r="G51" s="246">
-        <f>ROUND(19.4*$B$2,0)</f>
+        <f>SUM(F$24:F$25)*60231</f>
         <v/>
       </c>
       <c r="H51" s="246">
-        <f>ROUND(22.43*$B$2,0)</f>
+        <f>SUM(G$24:G$25)*65552</f>
         <v/>
       </c>
       <c r="I51" s="246">
-        <f>ROUND(21.8*$B$2,0)</f>
+        <f>SUM(H$24:H$25)*60210</f>
         <v/>
       </c>
       <c r="J51" s="246">
-        <f>ROUND(21.06*$B$2,0)</f>
+        <f>SUM(I$24:I$25)*55849</f>
         <v/>
       </c>
       <c r="K51" s="246">
-        <f>ROUND(21.36*$B$2,0)</f>
+        <f>SUM(J$24:J$25)*57094</f>
         <v/>
       </c>
       <c r="L51" s="246">
-        <f>ROUND(21.87*$B$2,0)</f>
+        <f>SUM(K$24:K$25)*60568</f>
         <v/>
       </c>
       <c r="M51" s="246">
-        <f>ROUND(21.65*$B$2,0)</f>
+        <f>SUM(L$24:L$25)*58837</f>
         <v/>
       </c>
       <c r="N51" s="246">
-        <f>ROUND(21.51*$B$2,0)</f>
+        <f>SUM(M$24:M$25)*58163</f>
         <v/>
       </c>
       <c r="O51" s="246">
-        <f>ROUND(21.47*$B$2,0)</f>
+        <f>SUM(N$24:N$25)*55242</f>
         <v/>
       </c>
       <c r="P51" s="246">
-        <f>ROUND(20.15*$B$2,0)</f>
+        <f>SUM(O$24:O$25)*46000</f>
         <v/>
       </c>
       <c r="Q51" s="246">
-        <f>ROUND(21.9*$B$2,0)</f>
+        <f>SUM(P$24:P$25)*58022</f>
         <v/>
       </c>
       <c r="R51" s="199">
@@ -18621,9 +18713,7 @@
     </row>
     <row r="52" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A52" s="225" t="n"/>
-      <c r="B52" s="179" t="n">
-        <v>9114120007</v>
-      </c>
+      <c r="B52" s="179" t="n"/>
       <c r="C52" s="182">
         <f>IFERROR(IF(VLOOKUP($B52,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B52,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -18837,7 +18927,10 @@
       <c r="K57" s="193" t="n"/>
       <c r="L57" s="193" t="n"/>
       <c r="M57" s="193" t="n"/>
-      <c r="N57" s="193" t="n"/>
+      <c r="N57" s="193">
+        <f>25*156600+2*170100</f>
+        <v/>
+      </c>
       <c r="O57" s="193" t="n"/>
       <c r="P57" s="193" t="n"/>
       <c r="Q57" s="193" t="n"/>
@@ -18909,18 +19002,45 @@
         <v/>
       </c>
       <c r="E59" s="244" t="n"/>
-      <c r="F59" s="193" t="n"/>
-      <c r="G59" s="193" t="n"/>
-      <c r="H59" s="193" t="n"/>
+      <c r="F59" s="193">
+        <f>1*152000</f>
+        <v/>
+      </c>
+      <c r="G59" s="193">
+        <f>1*152000</f>
+        <v/>
+      </c>
+      <c r="H59" s="193">
+        <f>2*152000</f>
+        <v/>
+      </c>
       <c r="I59" s="193" t="n"/>
       <c r="J59" s="193" t="n"/>
-      <c r="K59" s="193" t="n"/>
+      <c r="K59" s="193">
+        <f>1*152000</f>
+        <v/>
+      </c>
       <c r="L59" s="193" t="n"/>
-      <c r="M59" s="193" t="n"/>
-      <c r="N59" s="193" t="n"/>
-      <c r="O59" s="193" t="n"/>
-      <c r="P59" s="193" t="n"/>
-      <c r="Q59" s="193" t="n"/>
+      <c r="M59" s="193">
+        <f>1*152000</f>
+        <v/>
+      </c>
+      <c r="N59" s="193">
+        <f>1*152000</f>
+        <v/>
+      </c>
+      <c r="O59" s="193">
+        <f>2*152000</f>
+        <v/>
+      </c>
+      <c r="P59" s="193">
+        <f>1*152000</f>
+        <v/>
+      </c>
+      <c r="Q59" s="193">
+        <f>2*152000</f>
+        <v/>
+      </c>
       <c r="R59" s="199">
         <f>SUM(F59:Q59)</f>
         <v/>
@@ -19227,7 +19347,10 @@
       <c r="J67" s="193" t="n"/>
       <c r="K67" s="193" t="n"/>
       <c r="L67" s="193" t="n"/>
-      <c r="M67" s="193" t="n"/>
+      <c r="M67" s="193">
+        <f>27*107000</f>
+        <v/>
+      </c>
       <c r="N67" s="193" t="n"/>
       <c r="O67" s="193" t="n"/>
       <c r="P67" s="193" t="n"/>
@@ -19372,7 +19495,10 @@
       <c r="H71" s="193" t="n"/>
       <c r="I71" s="193" t="n"/>
       <c r="J71" s="193" t="n"/>
-      <c r="K71" s="193" t="n"/>
+      <c r="K71" s="193">
+        <f>27*56000</f>
+        <v/>
+      </c>
       <c r="L71" s="193" t="n"/>
       <c r="M71" s="193" t="n"/>
       <c r="N71" s="193" t="n"/>
@@ -20226,7 +20352,7 @@
     <row r="93" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A93" s="225" t="n"/>
       <c r="B93" s="179" t="n">
-        <v>5005016372</v>
+        <v>5005246281</v>
       </c>
       <c r="C93" s="182">
         <f>IFERROR(IF(VLOOKUP($B93,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B93,勘定科目!$A:$E,2,0)),"")</f>
@@ -20237,54 +20363,18 @@
         <v/>
       </c>
       <c r="E93" s="244" t="n"/>
-      <c r="F93" s="193">
-        <f>SUM(F$24:F$25)*1365</f>
-        <v/>
-      </c>
-      <c r="G93" s="193">
-        <f>SUM(F$24:F$25)*1284</f>
-        <v/>
-      </c>
-      <c r="H93" s="193">
-        <f>SUM(G$24:G$25)*1461</f>
-        <v/>
-      </c>
-      <c r="I93" s="193">
-        <f>SUM(H$24:H$25)*1517</f>
-        <v/>
-      </c>
-      <c r="J93" s="193">
-        <f>SUM(I$24:I$25)*1299</f>
-        <v/>
-      </c>
-      <c r="K93" s="193">
-        <f>SUM(J$24:J$25)*1328</f>
-        <v/>
-      </c>
-      <c r="L93" s="193">
-        <f>SUM(K$24:K$25)*1468</f>
-        <v/>
-      </c>
-      <c r="M93" s="193">
-        <f>SUM(L$24:L$25)*1426</f>
-        <v/>
-      </c>
-      <c r="N93" s="193">
-        <f>SUM(M$24:M$25)*1466</f>
-        <v/>
-      </c>
-      <c r="O93" s="193">
-        <f>SUM(N$24:N$25)*1339</f>
-        <v/>
-      </c>
-      <c r="P93" s="193">
-        <f>SUM(O$24:O$25)*803</f>
-        <v/>
-      </c>
-      <c r="Q93" s="193">
-        <f>SUM(P$24:P$25)*1462</f>
-        <v/>
-      </c>
+      <c r="F93" s="193" t="n"/>
+      <c r="G93" s="193" t="n"/>
+      <c r="H93" s="193" t="n"/>
+      <c r="I93" s="193" t="n"/>
+      <c r="J93" s="193" t="n"/>
+      <c r="K93" s="193" t="n"/>
+      <c r="L93" s="193" t="n"/>
+      <c r="M93" s="193" t="n"/>
+      <c r="N93" s="193" t="n"/>
+      <c r="O93" s="193" t="n"/>
+      <c r="P93" s="193" t="n"/>
+      <c r="Q93" s="193" t="n"/>
       <c r="R93" s="199">
         <f>SUM(F93:Q93)</f>
         <v/>
@@ -20297,9 +20387,7 @@
     </row>
     <row r="94" ht="13" customFormat="1" customHeight="1" s="207">
       <c r="A94" s="225" t="n"/>
-      <c r="B94" s="179" t="n">
-        <v>5005016372</v>
-      </c>
+      <c r="B94" s="179" t="n"/>
       <c r="C94" s="182">
         <f>IFERROR(IF(VLOOKUP($B94,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B94,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -20309,54 +20397,18 @@
         <v/>
       </c>
       <c r="E94" s="244" t="n"/>
-      <c r="F94" s="193">
-        <f>SUM(F$24:F$25)*18895</f>
-        <v/>
-      </c>
-      <c r="G94" s="193">
-        <f>SUM(F$24:F$25)*18117</f>
-        <v/>
-      </c>
-      <c r="H94" s="193">
-        <f>SUM(G$24:G$25)*20767</f>
-        <v/>
-      </c>
-      <c r="I94" s="193">
-        <f>SUM(H$24:H$25)*21675</f>
-        <v/>
-      </c>
-      <c r="J94" s="193">
-        <f>SUM(I$24:I$25)*17938</f>
-        <v/>
-      </c>
-      <c r="K94" s="193">
-        <f>SUM(J$24:J$25)*18894</f>
-        <v/>
-      </c>
-      <c r="L94" s="193">
-        <f>SUM(K$24:K$25)*20737</f>
-        <v/>
-      </c>
-      <c r="M94" s="193">
-        <f>SUM(L$24:L$25)*19781</f>
-        <v/>
-      </c>
-      <c r="N94" s="193">
-        <f>SUM(M$24:M$25)*20715</f>
-        <v/>
-      </c>
-      <c r="O94" s="193">
-        <f>SUM(N$24:N$25)*18874</f>
-        <v/>
-      </c>
-      <c r="P94" s="193">
-        <f>SUM(O$24:O$25)*11355</f>
-        <v/>
-      </c>
-      <c r="Q94" s="193">
-        <f>SUM(P$24:P$25)*20665</f>
-        <v/>
-      </c>
+      <c r="F94" s="193" t="n"/>
+      <c r="G94" s="193" t="n"/>
+      <c r="H94" s="193" t="n"/>
+      <c r="I94" s="193" t="n"/>
+      <c r="J94" s="193" t="n"/>
+      <c r="K94" s="193" t="n"/>
+      <c r="L94" s="193" t="n"/>
+      <c r="M94" s="193" t="n"/>
+      <c r="N94" s="193" t="n"/>
+      <c r="O94" s="193" t="n"/>
+      <c r="P94" s="193" t="n"/>
+      <c r="Q94" s="193" t="n"/>
       <c r="R94" s="199">
         <f>SUM(F94:Q94)</f>
         <v/>
@@ -25456,51 +25508,51 @@
       </c>
       <c r="E218" s="233" t="n"/>
       <c r="F218" s="234">
-        <f>22*152000</f>
+        <f>22*47000</f>
         <v/>
       </c>
       <c r="G218" s="234">
-        <f>22*152000</f>
+        <f>22*47000</f>
         <v/>
       </c>
       <c r="H218" s="234">
-        <f>26*152000</f>
+        <f>26*47000</f>
         <v/>
       </c>
       <c r="I218" s="234">
-        <f>27*152000</f>
+        <f>27*47000</f>
         <v/>
       </c>
       <c r="J218" s="234">
-        <f>27*152000</f>
+        <f>27*47000</f>
         <v/>
       </c>
       <c r="K218" s="234">
-        <f>27*152000</f>
+        <f>27*47000</f>
         <v/>
       </c>
       <c r="L218" s="234">
-        <f>27*152000</f>
+        <f>27*47000</f>
         <v/>
       </c>
       <c r="M218" s="234">
-        <f>27*152000</f>
+        <f>27*47000</f>
         <v/>
       </c>
       <c r="N218" s="234">
-        <f>27*152000</f>
+        <f>27*47000</f>
         <v/>
       </c>
       <c r="O218" s="234">
-        <f>28*152000</f>
+        <f>28*47000</f>
         <v/>
       </c>
       <c r="P218" s="234">
-        <f>28*152000</f>
+        <f>28*47000</f>
         <v/>
       </c>
       <c r="Q218" s="234">
-        <f>28*152000</f>
+        <f>28*47000</f>
         <v/>
       </c>
       <c r="R218" s="235">
@@ -25509,7 +25561,7 @@
       </c>
       <c r="S218" s="236" t="inlineStr">
         <is>
-          <t>Alloc: 誕生日会 Tiệc sinh nhật</t>
+          <t>Alloc: 金型用帽子（白）Mũ trắng tĩnh điện</t>
         </is>
       </c>
       <c r="T218" s="237" t="n"/>
@@ -25520,7 +25572,7 @@
     <row r="219" ht="13.5" customFormat="1" customHeight="1" s="207">
       <c r="A219" s="225" t="n"/>
       <c r="B219" s="178" t="n">
-        <v>5004086291</v>
+        <v>5005016372</v>
       </c>
       <c r="C219" s="231">
         <f>IFERROR(IF(VLOOKUP($B219,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B219,勘定科目!$A:$E,2,0)),"")</f>
@@ -25532,51 +25584,51 @@
       </c>
       <c r="E219" s="233" t="n"/>
       <c r="F219" s="234">
-        <f>22*47000</f>
+        <f>22*1</f>
         <v/>
       </c>
       <c r="G219" s="234">
-        <f>22*47000</f>
+        <f>22*1</f>
         <v/>
       </c>
       <c r="H219" s="234">
-        <f>26*47000</f>
+        <f>26*1</f>
         <v/>
       </c>
       <c r="I219" s="234">
-        <f>27*47000</f>
+        <f>27*1</f>
         <v/>
       </c>
       <c r="J219" s="234">
-        <f>27*47000</f>
+        <f>27*1</f>
         <v/>
       </c>
       <c r="K219" s="234">
-        <f>27*47000</f>
+        <f>27*1</f>
         <v/>
       </c>
       <c r="L219" s="234">
-        <f>27*47000</f>
+        <f>27*1</f>
         <v/>
       </c>
       <c r="M219" s="234">
-        <f>27*47000</f>
+        <f>27*1</f>
         <v/>
       </c>
       <c r="N219" s="234">
-        <f>27*47000</f>
+        <f>27*1</f>
         <v/>
       </c>
       <c r="O219" s="234">
-        <f>28*47000</f>
+        <f>28*1</f>
         <v/>
       </c>
       <c r="P219" s="234">
-        <f>28*47000</f>
+        <f>28*1</f>
         <v/>
       </c>
       <c r="Q219" s="234">
-        <f>28*47000</f>
+        <f>28*1</f>
         <v/>
       </c>
       <c r="R219" s="235">
@@ -25585,7 +25637,8 @@
       </c>
       <c r="S219" s="236" t="inlineStr">
         <is>
-          <t>Alloc: 金型用帽子（白）Mũ trắng tĩnh điện</t>
+          <t>Alloc: トイレットペーパー
+Giấy vệ sinh</t>
         </is>
       </c>
       <c r="T219" s="237" t="n"/>
@@ -25661,8 +25714,8 @@
       </c>
       <c r="S220" s="236" t="inlineStr">
         <is>
-          <t>Alloc: トイレットペーパー
-Giấy vệ sinh</t>
+          <t>Alloc: 手洗い洗剤
+Nước rửa tay</t>
         </is>
       </c>
       <c r="T220" s="237" t="n"/>
@@ -25673,7 +25726,7 @@
     <row r="221" ht="13.5" customFormat="1" customHeight="1" s="207">
       <c r="A221" s="225" t="n"/>
       <c r="B221" s="178" t="n">
-        <v>5005016372</v>
+        <v>5005056281</v>
       </c>
       <c r="C221" s="231">
         <f>IFERROR(IF(VLOOKUP($B221,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B221,勘定科目!$A:$E,2,0)),"")</f>
@@ -25738,8 +25791,7 @@
       </c>
       <c r="S221" s="236" t="inlineStr">
         <is>
-          <t>Alloc: 手洗い洗剤
-Nước rửa tay</t>
+          <t>Alloc: 食堂燃料費 Gas</t>
         </is>
       </c>
       <c r="T221" s="237" t="n"/>
@@ -25750,7 +25802,7 @@
     <row r="222" ht="13.5" customFormat="1" customHeight="1" s="207">
       <c r="A222" s="225" t="n"/>
       <c r="B222" s="178" t="n">
-        <v>5005056281</v>
+        <v>5005136281</v>
       </c>
       <c r="C222" s="231">
         <f>IFERROR(IF(VLOOKUP($B222,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B222,勘定科目!$A:$E,2,0)),"")</f>
@@ -25815,7 +25867,7 @@
       </c>
       <c r="S222" s="236" t="inlineStr">
         <is>
-          <t>Alloc: 食堂燃料費 Gas</t>
+          <t>Alloc: 社給携帯電話 Điện thoại di động công ty</t>
         </is>
       </c>
       <c r="T222" s="237" t="n"/>
@@ -25826,7 +25878,7 @@
     <row r="223" ht="13.5" customFormat="1" customHeight="1" s="207">
       <c r="A223" s="225" t="n"/>
       <c r="B223" s="178" t="n">
-        <v>5005136281</v>
+        <v>5005136291</v>
       </c>
       <c r="C223" s="231">
         <f>IFERROR(IF(VLOOKUP($B223,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B223,勘定科目!$A:$E,2,0)),"")</f>
@@ -25838,51 +25890,51 @@
       </c>
       <c r="E223" s="233" t="n"/>
       <c r="F223" s="234">
+        <f>20*1</f>
+        <v/>
+      </c>
+      <c r="G223" s="234">
+        <f>19*1</f>
+        <v/>
+      </c>
+      <c r="H223" s="234">
         <f>22*1</f>
         <v/>
       </c>
-      <c r="G223" s="234">
+      <c r="I223" s="234">
+        <f>23*1</f>
+        <v/>
+      </c>
+      <c r="J223" s="234">
+        <f>19*1</f>
+        <v/>
+      </c>
+      <c r="K223" s="234">
+        <f>20*1</f>
+        <v/>
+      </c>
+      <c r="L223" s="234">
         <f>22*1</f>
         <v/>
       </c>
-      <c r="H223" s="234">
-        <f>26*1</f>
-        <v/>
-      </c>
-      <c r="I223" s="234">
-        <f>27*1</f>
-        <v/>
-      </c>
-      <c r="J223" s="234">
-        <f>27*1</f>
-        <v/>
-      </c>
-      <c r="K223" s="234">
-        <f>27*1</f>
-        <v/>
-      </c>
-      <c r="L223" s="234">
-        <f>27*1</f>
-        <v/>
-      </c>
       <c r="M223" s="234">
-        <f>27*1</f>
+        <f>21*1</f>
         <v/>
       </c>
       <c r="N223" s="234">
-        <f>27*1</f>
+        <f>22*1</f>
         <v/>
       </c>
       <c r="O223" s="234">
-        <f>28*1</f>
+        <f>20*1</f>
         <v/>
       </c>
       <c r="P223" s="234">
-        <f>28*1</f>
+        <f>12*1</f>
         <v/>
       </c>
       <c r="Q223" s="234">
-        <f>28*1</f>
+        <f>22*1</f>
         <v/>
       </c>
       <c r="R223" s="235">
@@ -25891,7 +25943,7 @@
       </c>
       <c r="S223" s="236" t="inlineStr">
         <is>
-          <t>Alloc: 社給携帯電話 Điện thoại di động công ty</t>
+          <t>Alloc: 郵送 Chuyển phát nhanh</t>
         </is>
       </c>
       <c r="T223" s="237" t="n"/>
@@ -25902,7 +25954,7 @@
     <row r="224" ht="13.5" customFormat="1" customHeight="1" s="207">
       <c r="A224" s="225" t="n"/>
       <c r="B224" s="178" t="n">
-        <v>5005136291</v>
+        <v>5005246286</v>
       </c>
       <c r="C224" s="231">
         <f>IFERROR(IF(VLOOKUP($B224,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B224,勘定科目!$A:$E,2,0)),"")</f>
@@ -25914,51 +25966,51 @@
       </c>
       <c r="E224" s="233" t="n"/>
       <c r="F224" s="234">
-        <f>20*1</f>
+        <f>22*1</f>
         <v/>
       </c>
       <c r="G224" s="234">
-        <f>19*1</f>
+        <f>22*1</f>
         <v/>
       </c>
       <c r="H224" s="234">
-        <f>22*1</f>
+        <f>26*1</f>
         <v/>
       </c>
       <c r="I224" s="234">
-        <f>23*1</f>
+        <f>27*1</f>
         <v/>
       </c>
       <c r="J224" s="234">
-        <f>19*1</f>
+        <f>27*1</f>
         <v/>
       </c>
       <c r="K224" s="234">
-        <f>20*1</f>
+        <f>27*1</f>
         <v/>
       </c>
       <c r="L224" s="234">
-        <f>22*1</f>
+        <f>27*1</f>
         <v/>
       </c>
       <c r="M224" s="234">
-        <f>21*1</f>
+        <f>27*1</f>
         <v/>
       </c>
       <c r="N224" s="234">
-        <f>22*1</f>
+        <f>27*1</f>
         <v/>
       </c>
       <c r="O224" s="234">
-        <f>20*1</f>
+        <f>28*1</f>
         <v/>
       </c>
       <c r="P224" s="234">
-        <f>12*1</f>
+        <f>28*1</f>
         <v/>
       </c>
       <c r="Q224" s="234">
-        <f>22*1</f>
+        <f>28*1</f>
         <v/>
       </c>
       <c r="R224" s="235">
@@ -25967,7 +26019,7 @@
       </c>
       <c r="S224" s="236" t="inlineStr">
         <is>
-          <t>Alloc: 郵送 Chuyển phát nhanh</t>
+          <t>Alloc: 清掃費 Phí làm sạch</t>
         </is>
       </c>
       <c r="T224" s="237" t="n"/>
@@ -25977,9 +26029,7 @@
     </row>
     <row r="225" ht="13.5" customFormat="1" customHeight="1" s="207">
       <c r="A225" s="225" t="n"/>
-      <c r="B225" s="178" t="n">
-        <v>5005246286</v>
-      </c>
+      <c r="B225" s="178" t="n"/>
       <c r="C225" s="231">
         <f>IFERROR(IF(VLOOKUP($B225,勘定科目!$A:$H,HLOOKUP($E$5,勘定科目!$F$1:$H$2,2,0),0)="","",VLOOKUP($B225,勘定科目!$A:$E,2,0)),"")</f>
         <v/>
@@ -25989,63 +26039,23 @@
         <v/>
       </c>
       <c r="E225" s="233" t="n"/>
-      <c r="F225" s="234">
-        <f>22*1</f>
-        <v/>
-      </c>
-      <c r="G225" s="234">
-        <f>22*1</f>
-        <v/>
-      </c>
-      <c r="H225" s="234">
-        <f>26*1</f>
-        <v/>
-      </c>
-      <c r="I225" s="234">
-        <f>27*1</f>
-        <v/>
-      </c>
-      <c r="J225" s="234">
-        <f>27*1</f>
-        <v/>
-      </c>
-      <c r="K225" s="234">
-        <f>27*1</f>
-        <v/>
-      </c>
-      <c r="L225" s="234">
-        <f>27*1</f>
-        <v/>
-      </c>
-      <c r="M225" s="234">
-        <f>27*1</f>
-        <v/>
-      </c>
-      <c r="N225" s="234">
-        <f>27*1</f>
-        <v/>
-      </c>
-      <c r="O225" s="234">
-        <f>28*1</f>
-        <v/>
-      </c>
-      <c r="P225" s="234">
-        <f>28*1</f>
-        <v/>
-      </c>
-      <c r="Q225" s="234">
-        <f>28*1</f>
-        <v/>
-      </c>
+      <c r="F225" s="234" t="n"/>
+      <c r="G225" s="234" t="n"/>
+      <c r="H225" s="234" t="n"/>
+      <c r="I225" s="234" t="n"/>
+      <c r="J225" s="234" t="n"/>
+      <c r="K225" s="234" t="n"/>
+      <c r="L225" s="234" t="n"/>
+      <c r="M225" s="234" t="n"/>
+      <c r="N225" s="234" t="n"/>
+      <c r="O225" s="234" t="n"/>
+      <c r="P225" s="234" t="n"/>
+      <c r="Q225" s="234" t="n"/>
       <c r="R225" s="235">
         <f>SUM(F225:Q225)</f>
         <v/>
       </c>
-      <c r="S225" s="236" t="inlineStr">
-        <is>
-          <t>Alloc: 清掃費 Phí làm sạch</t>
-        </is>
-      </c>
+      <c r="S225" s="236" t="n"/>
       <c r="T225" s="237" t="n"/>
       <c r="U225" s="245" t="n"/>
       <c r="V225" s="245" t="n"/>

</xml_diff>